<commit_message>
v5-824 ADC calcs to low pr. thead
</commit_message>
<xml_diff>
--- a/HallFMBuggs.xlsx
+++ b/HallFMBuggs.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>R47 = 1k6, R45=4k7||100k = 4k25?</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Сделать 3V3, которые идут на пробник для питания EEPROM защищенными от кз</t>
+  </si>
+  <si>
+    <t>R71 make the same as R70, R59, R60</t>
   </si>
 </sst>
 </file>
@@ -373,7 +376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.44140625" customWidth="1"/>
@@ -460,6 +463,14 @@
         <v>9</v>
       </c>
     </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>46252</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>